<commit_message>
Actualizar cache, DWLT, pronostico y validacion Loreto
</commit_message>
<xml_diff>
--- a/outputs/metricas_dwlt_estaciones.xlsx
+++ b/outputs/metricas_dwlt_estaciones.xlsx
@@ -593,7 +593,7 @@
         <v>36.03138885531489</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1293773523170486</v>
+        <v>0.1293773523170485</v>
       </c>
       <c r="S2" t="n">
         <v>-0.7375148762927999</v>
@@ -812,13 +812,13 @@
         <v>1.911472491838996</v>
       </c>
       <c r="R5" t="n">
-        <v>0.3048585867839391</v>
+        <v>0.3048585867839389</v>
       </c>
       <c r="S5" t="n">
         <v>-0.1982415669926141</v>
       </c>
       <c r="T5" t="n">
-        <v>0.2802746963633374</v>
+        <v>0.2802746963633371</v>
       </c>
       <c r="U5" t="n">
         <v>6.7925</v>
@@ -885,13 +885,13 @@
         <v>1.494575642227743</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5089368211856863</v>
+        <v>0.5089368211856861</v>
       </c>
       <c r="S6" t="n">
         <v>0.07464598933846722</v>
       </c>
       <c r="T6" t="n">
-        <v>0.5050749116393327</v>
+        <v>0.5050749116393324</v>
       </c>
       <c r="U6" t="n">
         <v>6.109972296151311</v>
@@ -958,13 +958,13 @@
         <v>1.822552420274826</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8095836655428075</v>
+        <v>0.8095836655428076</v>
       </c>
       <c r="S7" t="n">
         <v>0.6303570018110684</v>
       </c>
       <c r="T7" t="n">
-        <v>0.7999405823947843</v>
+        <v>0.7999405823947844</v>
       </c>
       <c r="U7" t="n">
         <v>5.981758060466298</v>
@@ -1031,13 +1031,13 @@
         <v>1.920219108146032</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7617101500500636</v>
+        <v>0.761710150050064</v>
       </c>
       <c r="S8" t="n">
         <v>0.5361813343167756</v>
       </c>
       <c r="T8" t="n">
-        <v>0.7596994888028805</v>
+        <v>0.759699488802881</v>
       </c>
       <c r="U8" t="n">
         <v>6.53</v>
@@ -1104,13 +1104,13 @@
         <v>2.697554223649582</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3563464980514018</v>
+        <v>0.3563464980514016</v>
       </c>
       <c r="S9" t="n">
         <v>-0.1199845211161212</v>
       </c>
       <c r="T9" t="n">
-        <v>0.3354417007720807</v>
+        <v>0.3354417007720805</v>
       </c>
       <c r="U9" t="n">
         <v>10.1014171617984</v>
@@ -1250,13 +1250,13 @@
         <v>1.199886337673197</v>
       </c>
       <c r="R11" t="n">
-        <v>0.8289306355739895</v>
+        <v>0.8289306355739893</v>
       </c>
       <c r="S11" t="n">
         <v>0.6527307562356639</v>
       </c>
       <c r="T11" t="n">
-        <v>0.8272897533000165</v>
+        <v>0.8272897533000163</v>
       </c>
       <c r="U11" t="n">
         <v>5.281336733095788</v>
@@ -1323,13 +1323,13 @@
         <v>2.15549715055829</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8231978258912493</v>
+        <v>0.8231978258912499</v>
       </c>
       <c r="S12" t="n">
         <v>0.6484391411092192</v>
       </c>
       <c r="T12" t="n">
-        <v>0.8114941091534823</v>
+        <v>0.8114941091534829</v>
       </c>
       <c r="U12" t="n">
         <v>7.867834263294696</v>
@@ -1396,13 +1396,13 @@
         <v>2.285705332728494</v>
       </c>
       <c r="R13" t="n">
-        <v>0.7807763859794405</v>
+        <v>0.7807763859794399</v>
       </c>
       <c r="S13" t="n">
         <v>0.5650135915856762</v>
       </c>
       <c r="T13" t="n">
-        <v>0.7804109910934738</v>
+        <v>0.7804109910934731</v>
       </c>
       <c r="U13" t="n">
         <v>6.401922929815592</v>
@@ -1469,13 +1469,13 @@
         <v>2.700889385683155</v>
       </c>
       <c r="R14" t="n">
-        <v>0.7944316950721653</v>
+        <v>0.7944316950721657</v>
       </c>
       <c r="S14" t="n">
         <v>0.6086556188833412</v>
       </c>
       <c r="T14" t="n">
-        <v>0.7858592938199808</v>
+        <v>0.7858592938199812</v>
       </c>
       <c r="U14" t="n">
         <v>8.388284851374982</v>
@@ -1615,13 +1615,13 @@
         <v>2.579583230291027</v>
       </c>
       <c r="R16" t="n">
-        <v>0.5181653642573085</v>
+        <v>0.5181653642573086</v>
       </c>
       <c r="S16" t="n">
         <v>0.01527028269559583</v>
       </c>
       <c r="T16" t="n">
-        <v>0.5148572754275724</v>
+        <v>0.5148572754275725</v>
       </c>
       <c r="U16" t="n">
         <v>3.950317923339689</v>
@@ -1688,13 +1688,13 @@
         <v>1.488644272773963</v>
       </c>
       <c r="R17" t="n">
-        <v>0.5997299970012603</v>
+        <v>0.5997299970012602</v>
       </c>
       <c r="S17" t="n">
         <v>0.2151241668148857</v>
       </c>
       <c r="T17" t="n">
-        <v>0.5967713101904909</v>
+        <v>0.5967713101904908</v>
       </c>
       <c r="U17" t="n">
         <v>4.866268240618501</v>
@@ -1761,13 +1761,13 @@
         <v>2.750576503734912</v>
       </c>
       <c r="R18" t="n">
-        <v>0.7262145542217276</v>
+        <v>0.7262145542217279</v>
       </c>
       <c r="S18" t="n">
         <v>0.4688815464657763</v>
       </c>
       <c r="T18" t="n">
-        <v>0.6791774910414113</v>
+        <v>0.6791774910414116</v>
       </c>
       <c r="U18" t="n">
         <v>7.962271702191409</v>

</xml_diff>

<commit_message>
Actualizar cache, DWLT, pronostico, historico y validacion Loreto
</commit_message>
<xml_diff>
--- a/outputs/metricas_dwlt_estaciones.xlsx
+++ b/outputs/metricas_dwlt_estaciones.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -603,40 +603,40 @@
         <v>118.97</v>
       </c>
       <c r="O2" t="n">
-        <v>2.26</v>
+        <v>1.843123209169055</v>
       </c>
       <c r="P2" t="n">
-        <v>95.32108891119333</v>
+        <v>102.8805069991831</v>
       </c>
       <c r="Q2" t="n">
-        <v>118.38</v>
+        <v>118.8919225199131</v>
       </c>
       <c r="R2" t="n">
-        <v>-7.560093533675002</v>
+        <v>-0.0006754456851761013</v>
       </c>
       <c r="S2" t="n">
-        <v>22.67654031248787</v>
+        <v>17.76440495292452</v>
       </c>
       <c r="T2" t="n">
-        <v>31.5619114901981</v>
+        <v>36.12789924823703</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1346527683752431</v>
+        <v>0.1290306914977253</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.3250996326126141</v>
+        <v>-0.7362304019696044</v>
       </c>
       <c r="W2" t="n">
-        <v>0.06424909254152456</v>
+        <v>0.1290245036301099</v>
       </c>
       <c r="X2" t="n">
-        <v>87.20004320936965</v>
+        <v>58.62662276669903</v>
       </c>
       <c r="Y2" t="n">
-        <v>91.79737419881558</v>
+        <v>105.0571713563318</v>
       </c>
       <c r="Z2" t="n">
-        <v>103.6245390887595</v>
+        <v>110.9100723655944</v>
       </c>
     </row>
     <row r="3">
@@ -650,7 +650,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -689,40 +689,40 @@
         <v>11.07</v>
       </c>
       <c r="O3" t="n">
-        <v>0.01185120904911286</v>
+        <v>0.01756303724928367</v>
       </c>
       <c r="P3" t="n">
-        <v>4.955393767974834</v>
+        <v>4.960253486539629</v>
       </c>
       <c r="Q3" t="n">
         <v>11.07</v>
       </c>
       <c r="R3" t="n">
-        <v>0.04880321841846751</v>
+        <v>0.05366293698326334</v>
       </c>
       <c r="S3" t="n">
-        <v>1.35378970316816</v>
+        <v>1.350867190817886</v>
       </c>
       <c r="T3" t="n">
-        <v>1.729651006670732</v>
+        <v>1.725583767663616</v>
       </c>
       <c r="U3" t="n">
-        <v>0.7784584130179306</v>
+        <v>0.7794857527669876</v>
       </c>
       <c r="V3" t="n">
-        <v>0.5643785245295188</v>
+        <v>0.5664248257801628</v>
       </c>
       <c r="W3" t="n">
-        <v>0.7774743743353822</v>
+        <v>0.7784293892948898</v>
       </c>
       <c r="X3" t="n">
-        <v>2.726657362903647</v>
+        <v>2.712659863698741</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.1287505843467</v>
+        <v>3.151962644367367</v>
       </c>
       <c r="Z3" t="n">
-        <v>3.673135756733777</v>
+        <v>3.734334088493765</v>
       </c>
     </row>
     <row r="4">
@@ -736,7 +736,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -775,40 +775,40 @@
         <v>12.93</v>
       </c>
       <c r="O4" t="n">
-        <v>0.5052697142338819</v>
+        <v>0.3662633451957295</v>
       </c>
       <c r="P4" t="n">
-        <v>7.237698632435657</v>
+        <v>7.247986940912678</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.79092695825988</v>
+        <v>12.72990889978977</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3186412994936734</v>
+        <v>0.3289296079706954</v>
       </c>
       <c r="S4" t="n">
-        <v>1.289777543834538</v>
+        <v>1.294332688333304</v>
       </c>
       <c r="T4" t="n">
-        <v>1.677310713563687</v>
+        <v>1.684282371589636</v>
       </c>
       <c r="U4" t="n">
-        <v>0.8680610691971837</v>
+        <v>0.8674230549645812</v>
       </c>
       <c r="V4" t="n">
-        <v>0.7392154023818902</v>
+        <v>0.7370430207935936</v>
       </c>
       <c r="W4" t="n">
-        <v>0.8471523306135846</v>
+        <v>0.8471326096588474</v>
       </c>
       <c r="X4" t="n">
-        <v>4.659168758156628</v>
+        <v>4.564022737736554</v>
       </c>
       <c r="Y4" t="n">
-        <v>4.782537555386879</v>
+        <v>4.704556034058134</v>
       </c>
       <c r="Z4" t="n">
-        <v>4.87826428304801</v>
+        <v>4.850516014234875</v>
       </c>
     </row>
     <row r="5">
@@ -822,7 +822,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -861,40 +861,40 @@
         <v>10.6125</v>
       </c>
       <c r="O5" t="n">
-        <v>2.074263578685523</v>
+        <v>1.616683937823834</v>
       </c>
       <c r="P5" t="n">
-        <v>6.923698638566593</v>
+        <v>7.018400774846545</v>
       </c>
       <c r="Q5" t="n">
-        <v>10.02216567852482</v>
+        <v>10.19100035038542</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1933108441825349</v>
+        <v>0.2880129804624863</v>
       </c>
       <c r="S5" t="n">
-        <v>1.446668089612012</v>
+        <v>1.482517678733487</v>
       </c>
       <c r="T5" t="n">
-        <v>1.844871649448231</v>
+        <v>1.911088301545514</v>
       </c>
       <c r="U5" t="n">
-        <v>0.2963057040290977</v>
+        <v>0.3047869471349391</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.1165617051816392</v>
+        <v>-0.198152015826023</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2473718084235209</v>
+        <v>0.280195644835217</v>
       </c>
       <c r="X5" t="n">
-        <v>6.655022829612451</v>
+        <v>6.583047424731074</v>
       </c>
       <c r="Y5" t="n">
-        <v>6.819912168590496</v>
+        <v>6.698516263439359</v>
       </c>
       <c r="Z5" t="n">
-        <v>7.020748537994402</v>
+        <v>6.900139837360185</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +908,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -947,40 +947,40 @@
         <v>10.01</v>
       </c>
       <c r="O6" t="n">
-        <v>1.18</v>
+        <v>1.33253223495702</v>
       </c>
       <c r="P6" t="n">
-        <v>5.585509222811802</v>
+        <v>5.586612252363356</v>
       </c>
       <c r="Q6" t="n">
         <v>10.01</v>
       </c>
       <c r="R6" t="n">
-        <v>0.00277796312461025</v>
+        <v>0.003880992676163806</v>
       </c>
       <c r="S6" t="n">
-        <v>1.162507910021187</v>
+        <v>1.156005201629343</v>
       </c>
       <c r="T6" t="n">
-        <v>1.500686020616032</v>
+        <v>1.494185346244633</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5076689963535944</v>
+        <v>0.5089834682959363</v>
       </c>
       <c r="V6" t="n">
-        <v>0.06661454802383027</v>
+        <v>0.0746835150260281</v>
       </c>
       <c r="W6" t="n">
-        <v>0.5045872899967179</v>
+        <v>0.5051305807576973</v>
       </c>
       <c r="X6" t="n">
-        <v>5.726760030246275</v>
+        <v>5.734153605288033</v>
       </c>
       <c r="Y6" t="n">
-        <v>5.944611091641512</v>
+        <v>5.961456061839657</v>
       </c>
       <c r="Z6" t="n">
-        <v>6.177788607260648</v>
+        <v>6.171095644044707</v>
       </c>
     </row>
     <row r="7">
@@ -994,7 +994,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1033,40 +1033,40 @@
         <v>15.14</v>
       </c>
       <c r="O7" t="n">
-        <v>1.098396014558873</v>
+        <v>0.6453438395415473</v>
       </c>
       <c r="P7" t="n">
-        <v>8.09313870584355</v>
+        <v>8.116958313273042</v>
       </c>
       <c r="Q7" t="n">
-        <v>13.93778665249157</v>
+        <v>14.26297827610371</v>
       </c>
       <c r="R7" t="n">
-        <v>0.2125701449004903</v>
+        <v>0.2363897523299814</v>
       </c>
       <c r="S7" t="n">
-        <v>1.421964885303135</v>
+        <v>1.444727910070825</v>
       </c>
       <c r="T7" t="n">
-        <v>1.794874374992412</v>
+        <v>1.824450631234724</v>
       </c>
       <c r="U7" t="n">
-        <v>0.8123781964764707</v>
+        <v>0.8089378617134542</v>
       </c>
       <c r="V7" t="n">
-        <v>0.6412221059864125</v>
+        <v>0.6293006761981014</v>
       </c>
       <c r="W7" t="n">
-        <v>0.7977428869926722</v>
+        <v>0.7992692537450868</v>
       </c>
       <c r="X7" t="n">
-        <v>5.425722835462518</v>
+        <v>5.431714396783157</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.780232245256398</v>
+        <v>5.792866714554191</v>
       </c>
       <c r="Z7" t="n">
-        <v>6.275026515803463</v>
+        <v>6.23841994793755</v>
       </c>
     </row>
     <row r="8">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1119,40 +1119,40 @@
         <v>14.03</v>
       </c>
       <c r="O8" t="n">
-        <v>1.106025794920669</v>
+        <v>0.5109074733096085</v>
       </c>
       <c r="P8" t="n">
-        <v>7.66001777880603</v>
+        <v>7.680453857551946</v>
       </c>
       <c r="Q8" t="n">
         <v>14.03</v>
       </c>
       <c r="R8" t="n">
-        <v>0.04349833015191976</v>
+        <v>0.06393440889783572</v>
       </c>
       <c r="S8" t="n">
-        <v>1.502488439761694</v>
+        <v>1.477664670365433</v>
       </c>
       <c r="T8" t="n">
-        <v>1.961806731289439</v>
+        <v>1.920049134906619</v>
       </c>
       <c r="U8" t="n">
-        <v>0.7529672973981634</v>
+        <v>0.7616658933081911</v>
       </c>
       <c r="V8" t="n">
-        <v>0.5156645002114295</v>
+        <v>0.5360634946554466</v>
       </c>
       <c r="W8" t="n">
-        <v>0.7520042259461893</v>
+        <v>0.7596843787542078</v>
       </c>
       <c r="X8" t="n">
-        <v>5.867810134768883</v>
+        <v>5.824999999999999</v>
       </c>
       <c r="Y8" t="n">
-        <v>6.267092667943198</v>
+        <v>6.246853956131093</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.796228742714516</v>
+        <v>6.819118199903117</v>
       </c>
     </row>
     <row r="9">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1208,37 +1208,37 @@
         <v>4.255000000000001</v>
       </c>
       <c r="P9" t="n">
-        <v>10.74252406872358</v>
+        <v>10.61997044208291</v>
       </c>
       <c r="Q9" t="n">
-        <v>23.3656067150359</v>
+        <v>14.31645908761767</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4374645289858261</v>
+        <v>0.3149109023451558</v>
       </c>
       <c r="S9" t="n">
-        <v>2.151324667917073</v>
+        <v>2.051512150992676</v>
       </c>
       <c r="T9" t="n">
-        <v>2.874361963841202</v>
+        <v>2.697239871879806</v>
       </c>
       <c r="U9" t="n">
-        <v>0.3308464323914269</v>
+        <v>0.3565374589986294</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.2716118563734509</v>
+        <v>-0.1197235079364318</v>
       </c>
       <c r="W9" t="n">
-        <v>0.3251872978382808</v>
+        <v>0.3356971120163307</v>
       </c>
       <c r="X9" t="n">
-        <v>10.02178617217574</v>
+        <v>9.985830193984139</v>
       </c>
       <c r="Y9" t="n">
-        <v>10.17595530833749</v>
+        <v>10.14751528255746</v>
       </c>
       <c r="Z9" t="n">
-        <v>10.29171099478866</v>
+        <v>10.26376587323174</v>
       </c>
     </row>
     <row r="10">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1291,40 +1291,40 @@
         <v>10.15</v>
       </c>
       <c r="O10" t="n">
-        <v>0.4490779286658197</v>
+        <v>0.8401943005181348</v>
       </c>
       <c r="P10" t="n">
-        <v>5.218764597108932</v>
+        <v>5.218400961295386</v>
       </c>
       <c r="Q10" t="n">
         <v>9.94</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.02710672482178227</v>
+        <v>-0.02747036063532915</v>
       </c>
       <c r="S10" t="n">
-        <v>1.160595399939246</v>
+        <v>1.158007997174354</v>
       </c>
       <c r="T10" t="n">
-        <v>1.481666993510793</v>
+        <v>1.476930319096901</v>
       </c>
       <c r="U10" t="n">
-        <v>0.4297098221582691</v>
+        <v>0.4295536771628595</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.08914771699724922</v>
+        <v>-0.0821951534883727</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4277215945596142</v>
+        <v>0.4269447872355635</v>
       </c>
       <c r="X10" t="n">
-        <v>4.44803834147273</v>
+        <v>4.448242129297602</v>
       </c>
       <c r="Y10" t="n">
-        <v>4.636119518503951</v>
+        <v>4.673430666105889</v>
       </c>
       <c r="Z10" t="n">
-        <v>4.799240421107129</v>
+        <v>4.84023487544484</v>
       </c>
     </row>
     <row r="11">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1377,40 +1377,40 @@
         <v>19.1775</v>
       </c>
       <c r="O11" t="n">
-        <v>2.365562336565191</v>
+        <v>2.204850111028867</v>
       </c>
       <c r="P11" t="n">
-        <v>7.711831118294073</v>
+        <v>7.667681588419747</v>
       </c>
       <c r="Q11" t="n">
-        <v>13.28491592512375</v>
+        <v>16.78594914040094</v>
       </c>
       <c r="R11" t="n">
-        <v>0.2165802679539373</v>
+        <v>0.1724307380796102</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9626458364738362</v>
+        <v>0.9154934511717434</v>
       </c>
       <c r="T11" t="n">
-        <v>1.342385845624896</v>
+        <v>1.198712428655893</v>
       </c>
       <c r="U11" t="n">
-        <v>0.7909457516916999</v>
+        <v>0.8292281531466016</v>
       </c>
       <c r="V11" t="n">
-        <v>0.5654800662863657</v>
+        <v>0.6535145573915913</v>
       </c>
       <c r="W11" t="n">
-        <v>0.7886250637390947</v>
+        <v>0.8275572060890022</v>
       </c>
       <c r="X11" t="n">
-        <v>4.915233112762575</v>
+        <v>4.926820442691524</v>
       </c>
       <c r="Y11" t="n">
-        <v>5.160518194367339</v>
+        <v>5.154828226624991</v>
       </c>
       <c r="Z11" t="n">
-        <v>5.34356916065347</v>
+        <v>5.339127765106988</v>
       </c>
     </row>
     <row r="12">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1463,40 +1463,40 @@
         <v>16.215</v>
       </c>
       <c r="O12" t="n">
-        <v>2.953822385664691</v>
+        <v>2.860487544483985</v>
       </c>
       <c r="P12" t="n">
-        <v>10.01642806999197</v>
+        <v>10.03206015250905</v>
       </c>
       <c r="Q12" t="n">
-        <v>16.13</v>
+        <v>16.20563653352021</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3979510674079892</v>
+        <v>0.4135831499250696</v>
       </c>
       <c r="S12" t="n">
-        <v>1.682949594310256</v>
+        <v>1.695183761897019</v>
       </c>
       <c r="T12" t="n">
-        <v>2.13777110892555</v>
+        <v>2.154633561662434</v>
       </c>
       <c r="U12" t="n">
-        <v>0.8253777564634406</v>
+        <v>0.8231449621794996</v>
       </c>
       <c r="V12" t="n">
-        <v>0.6539368807194608</v>
+        <v>0.6484559499651469</v>
       </c>
       <c r="W12" t="n">
-        <v>0.8134780543479637</v>
+        <v>0.8113194274977851</v>
       </c>
       <c r="X12" t="n">
-        <v>7.329069077238741</v>
+        <v>7.327769604254384</v>
       </c>
       <c r="Y12" t="n">
-        <v>7.719598520648679</v>
+        <v>7.688770065273216</v>
       </c>
       <c r="Z12" t="n">
-        <v>8.022530992927182</v>
+        <v>8.015356698101943</v>
       </c>
     </row>
     <row r="13">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1549,40 +1549,40 @@
         <v>34.0025</v>
       </c>
       <c r="O13" t="n">
-        <v>0.8778757365545877</v>
+        <v>0.91</v>
       </c>
       <c r="P13" t="n">
-        <v>8.211816165527123</v>
+        <v>8.204022517489584</v>
       </c>
       <c r="Q13" t="n">
-        <v>19.64109372411599</v>
+        <v>14.32</v>
       </c>
       <c r="R13" t="n">
-        <v>0.07747028292276292</v>
+        <v>0.06967663488522495</v>
       </c>
       <c r="S13" t="n">
-        <v>1.786781978331799</v>
+        <v>1.759977967731633</v>
       </c>
       <c r="T13" t="n">
-        <v>2.321771379560974</v>
+        <v>2.285358155561822</v>
       </c>
       <c r="U13" t="n">
-        <v>0.7761818370206299</v>
+        <v>0.7806980901130567</v>
       </c>
       <c r="V13" t="n">
-        <v>0.5509625937169469</v>
+        <v>0.5649369937042079</v>
       </c>
       <c r="W13" t="n">
-        <v>0.7759703359358315</v>
+        <v>0.7803386521161693</v>
       </c>
       <c r="X13" t="n">
-        <v>6.290375714976573</v>
+        <v>6.175338062833483</v>
       </c>
       <c r="Y13" t="n">
-        <v>6.4632821178661</v>
+        <v>6.330156553077177</v>
       </c>
       <c r="Z13" t="n">
-        <v>6.634535108837767</v>
+        <v>6.512216211567904</v>
       </c>
     </row>
     <row r="14">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1635,40 +1635,40 @@
         <v>30.745</v>
       </c>
       <c r="O14" t="n">
-        <v>4.975807364456732</v>
+        <v>4.682413027387121</v>
       </c>
       <c r="P14" t="n">
-        <v>11.83304847267143</v>
+        <v>11.82552192549244</v>
       </c>
       <c r="Q14" t="n">
-        <v>21.27195770556229</v>
+        <v>21.32952932657494</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.1308334247148275</v>
+        <v>-0.1383599718938091</v>
       </c>
       <c r="S14" t="n">
-        <v>2.043091105259739</v>
+        <v>2.052549934730245</v>
       </c>
       <c r="T14" t="n">
-        <v>2.658841148422919</v>
+        <v>2.698059965267305</v>
       </c>
       <c r="U14" t="n">
-        <v>0.8009818143304313</v>
+        <v>0.794744098747145</v>
       </c>
       <c r="V14" t="n">
-        <v>0.6207458960241264</v>
+        <v>0.6094751250813673</v>
       </c>
       <c r="W14" t="n">
-        <v>0.7924356139012816</v>
+        <v>0.7858579931677233</v>
       </c>
       <c r="X14" t="n">
-        <v>8.054630084232455</v>
+        <v>8.171810589981328</v>
       </c>
       <c r="Y14" t="n">
-        <v>8.405661885264568</v>
+        <v>8.296913495104311</v>
       </c>
       <c r="Z14" t="n">
-        <v>8.794140384354014</v>
+        <v>8.389419204380809</v>
       </c>
     </row>
     <row r="15">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1721,40 +1721,40 @@
         <v>131.9</v>
       </c>
       <c r="O15" t="n">
-        <v>0.5804528488899593</v>
+        <v>0.5268935553946416</v>
       </c>
       <c r="P15" t="n">
-        <v>9.376418874129996</v>
+        <v>8.66355542641087</v>
       </c>
       <c r="Q15" t="n">
-        <v>119.6249412815277</v>
+        <v>131.7868211440985</v>
       </c>
       <c r="R15" t="n">
-        <v>0.9670057190097701</v>
+        <v>0.2541422712906439</v>
       </c>
       <c r="S15" t="n">
-        <v>4.183232496061627</v>
+        <v>3.53679365639656</v>
       </c>
       <c r="T15" t="n">
-        <v>11.62063429137672</v>
+        <v>11.06520679939195</v>
       </c>
       <c r="U15" t="n">
-        <v>0.03397869450270663</v>
+        <v>0.04964511346769675</v>
       </c>
       <c r="V15" t="n">
-        <v>-0.7612938482567244</v>
+        <v>-0.596949638179824</v>
       </c>
       <c r="W15" t="n">
-        <v>0.02204797432166528</v>
+        <v>0.03288895518929591</v>
       </c>
       <c r="X15" t="n">
-        <v>10.88721575317732</v>
+        <v>10.81954001023077</v>
       </c>
       <c r="Y15" t="n">
-        <v>11.3663279587366</v>
+        <v>11.35346457164039</v>
       </c>
       <c r="Z15" t="n">
-        <v>11.84771123132677</v>
+        <v>11.81034798284707</v>
       </c>
     </row>
     <row r="16">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1807,40 +1807,40 @@
         <v>12.23</v>
       </c>
       <c r="O16" t="n">
-        <v>1.467998349796847</v>
+        <v>1.395549592894153</v>
       </c>
       <c r="P16" t="n">
-        <v>6.927568537229587</v>
+        <v>6.954939778501083</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.11960615380856</v>
+        <v>12.15738414192614</v>
       </c>
       <c r="R16" t="n">
-        <v>0.3444351315896731</v>
+        <v>0.3718063728611686</v>
       </c>
       <c r="S16" t="n">
-        <v>1.971989331991212</v>
+        <v>2.040734871266995</v>
       </c>
       <c r="T16" t="n">
-        <v>2.479912148565002</v>
+        <v>2.579822443878717</v>
       </c>
       <c r="U16" t="n">
-        <v>0.5334811347299319</v>
+        <v>0.518110315037839</v>
       </c>
       <c r="V16" t="n">
-        <v>0.08989699853024857</v>
+        <v>0.01508763950890413</v>
       </c>
       <c r="W16" t="n">
-        <v>0.5283441202157942</v>
+        <v>0.5148113820469902</v>
       </c>
       <c r="X16" t="n">
-        <v>3.370754207582492</v>
+        <v>3.256802654783871</v>
       </c>
       <c r="Y16" t="n">
-        <v>4.201833754927192</v>
+        <v>4.216359069012279</v>
       </c>
       <c r="Z16" t="n">
-        <v>5.238002578823759</v>
+        <v>5.085508762630371</v>
       </c>
     </row>
     <row r="17">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1893,40 +1893,40 @@
         <v>18.4925</v>
       </c>
       <c r="O17" t="n">
-        <v>1.923435659174772</v>
+        <v>1.826106587712805</v>
       </c>
       <c r="P17" t="n">
-        <v>6.724897375817505</v>
+        <v>6.69644383013072</v>
       </c>
       <c r="Q17" t="n">
-        <v>13.28173148390984</v>
+        <v>14.92774999999984</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2230450037825492</v>
+        <v>0.1945914580957638</v>
       </c>
       <c r="S17" t="n">
-        <v>1.08906507232978</v>
+        <v>1.098093270421765</v>
       </c>
       <c r="T17" t="n">
-        <v>1.478031836906768</v>
+        <v>1.4879502314557</v>
       </c>
       <c r="U17" t="n">
-        <v>0.6081939627971509</v>
+        <v>0.6007892903475741</v>
       </c>
       <c r="V17" t="n">
-        <v>0.2274777624876755</v>
+        <v>0.2170748890872708</v>
       </c>
       <c r="W17" t="n">
-        <v>0.604815791493112</v>
+        <v>0.5978707599418338</v>
       </c>
       <c r="X17" t="n">
-        <v>4.477105858498857</v>
+        <v>4.407509507712392</v>
       </c>
       <c r="Y17" t="n">
-        <v>5.447938047516743</v>
+        <v>5.481337855009455</v>
       </c>
       <c r="Z17" t="n">
-        <v>6.238323917510907</v>
+        <v>6.282784819998072</v>
       </c>
     </row>
     <row r="18">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>histograma_cdf_mensual_optimizado</t>
+          <t>cdf_empirica_mensual_ordenada</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1979,40 +1979,40 @@
         <v>24.5875</v>
       </c>
       <c r="O18" t="n">
-        <v>4.731988859052884</v>
+        <v>4.725023439427584</v>
       </c>
       <c r="P18" t="n">
-        <v>11.16594572584583</v>
+        <v>11.1579530595688</v>
       </c>
       <c r="Q18" t="n">
-        <v>17.5154399668629</v>
+        <v>17.53862298528381</v>
       </c>
       <c r="R18" t="n">
-        <v>0.7910232614702994</v>
+        <v>0.783030595193274</v>
       </c>
       <c r="S18" t="n">
-        <v>2.037989632240806</v>
+        <v>2.035657657160924</v>
       </c>
       <c r="T18" t="n">
-        <v>2.759216533459643</v>
+        <v>2.754661476283585</v>
       </c>
       <c r="U18" t="n">
-        <v>0.7252654719829723</v>
+        <v>0.7262807610849884</v>
       </c>
       <c r="V18" t="n">
-        <v>0.4674592809286297</v>
+        <v>0.4692161210425043</v>
       </c>
       <c r="W18" t="n">
-        <v>0.6763526951715143</v>
+        <v>0.6790166987374697</v>
       </c>
       <c r="X18" t="n">
-        <v>7.883441301049346</v>
+        <v>7.820460753846925</v>
       </c>
       <c r="Y18" t="n">
-        <v>8.025719050129879</v>
+        <v>7.920922767604085</v>
       </c>
       <c r="Z18" t="n">
-        <v>8.101192844461115</v>
+        <v>7.979100294050045</v>
       </c>
     </row>
   </sheetData>
@@ -2090,13 +2090,13 @@
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>7.883441301049346</v>
+        <v>7.820460753846925</v>
       </c>
       <c r="G2" t="n">
-        <v>8.025719050129879</v>
+        <v>7.920922767604085</v>
       </c>
       <c r="H2" t="n">
-        <v>8.101192844461115</v>
+        <v>7.979100294050045</v>
       </c>
     </row>
     <row r="3">
@@ -2118,13 +2118,13 @@
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>5.726760030246275</v>
+        <v>5.734153605288033</v>
       </c>
       <c r="G3" t="n">
-        <v>5.944611091641513</v>
+        <v>5.961456061839657</v>
       </c>
       <c r="H3" t="n">
-        <v>6.177788607260648</v>
+        <v>6.171095644044707</v>
       </c>
     </row>
     <row r="4">
@@ -2146,13 +2146,13 @@
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>4.44803834147273</v>
+        <v>4.448242129297602</v>
       </c>
       <c r="G4" t="n">
-        <v>4.636119518503951</v>
+        <v>4.673430666105889</v>
       </c>
       <c r="H4" t="n">
-        <v>4.799240421107129</v>
+        <v>4.84023487544484</v>
       </c>
     </row>
     <row r="5">
@@ -2174,13 +2174,13 @@
         <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>10.88721575317732</v>
+        <v>10.81954001023077</v>
       </c>
       <c r="G5" t="n">
-        <v>11.3663279587366</v>
+        <v>11.35346457164039</v>
       </c>
       <c r="H5" t="n">
-        <v>11.84771123132677</v>
+        <v>11.81034798284707</v>
       </c>
     </row>
     <row r="6">
@@ -2202,13 +2202,13 @@
         <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>87.20004320936965</v>
+        <v>58.62662276669903</v>
       </c>
       <c r="G6" t="n">
-        <v>91.79737419881558</v>
+        <v>105.0571713563318</v>
       </c>
       <c r="H6" t="n">
-        <v>103.6245390887595</v>
+        <v>110.9100723655944</v>
       </c>
     </row>
     <row r="7">
@@ -2230,13 +2230,13 @@
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>8.054630084232455</v>
+        <v>8.171810589981328</v>
       </c>
       <c r="G7" t="n">
-        <v>8.405661885264564</v>
+        <v>8.296913495104311</v>
       </c>
       <c r="H7" t="n">
-        <v>8.794140384354014</v>
+        <v>8.389419204380809</v>
       </c>
     </row>
     <row r="8">
@@ -2258,13 +2258,13 @@
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>7.329069077238741</v>
+        <v>7.327769604254384</v>
       </c>
       <c r="G8" t="n">
-        <v>7.719598520648679</v>
+        <v>7.688770065273216</v>
       </c>
       <c r="H8" t="n">
-        <v>8.022530992927182</v>
+        <v>8.015356698101943</v>
       </c>
     </row>
     <row r="9">
@@ -2286,13 +2286,13 @@
         <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>4.915233112762575</v>
+        <v>4.926820442691524</v>
       </c>
       <c r="G9" t="n">
-        <v>5.160518194367338</v>
+        <v>5.154828226624991</v>
       </c>
       <c r="H9" t="n">
-        <v>5.34356916065347</v>
+        <v>5.339127765106988</v>
       </c>
     </row>
     <row r="10">
@@ -2314,13 +2314,13 @@
         <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>5.425722835462518</v>
+        <v>5.431714396783157</v>
       </c>
       <c r="G10" t="n">
-        <v>5.780232245256398</v>
+        <v>5.792866714554192</v>
       </c>
       <c r="H10" t="n">
-        <v>6.275026515803463</v>
+        <v>6.23841994793755</v>
       </c>
     </row>
     <row r="11">
@@ -2342,13 +2342,13 @@
         <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>3.370754207582492</v>
+        <v>3.256802654783871</v>
       </c>
       <c r="G11" t="n">
-        <v>4.201833754927192</v>
+        <v>4.216359069012278</v>
       </c>
       <c r="H11" t="n">
-        <v>5.238002578823759</v>
+        <v>5.085508762630371</v>
       </c>
     </row>
     <row r="12">
@@ -2370,13 +2370,13 @@
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>6.290375714976573</v>
+        <v>6.175338062833483</v>
       </c>
       <c r="G12" t="n">
-        <v>6.4632821178661</v>
+        <v>6.330156553077177</v>
       </c>
       <c r="H12" t="n">
-        <v>6.634535108837767</v>
+        <v>6.512216211567904</v>
       </c>
     </row>
     <row r="13">
@@ -2398,13 +2398,13 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>10.02178617217574</v>
+        <v>9.985830193984139</v>
       </c>
       <c r="G13" t="n">
-        <v>10.17595530833749</v>
+        <v>10.14751528255746</v>
       </c>
       <c r="H13" t="n">
-        <v>10.29171099478866</v>
+        <v>10.26376587323174</v>
       </c>
     </row>
     <row r="14">
@@ -2426,13 +2426,13 @@
         <v>10</v>
       </c>
       <c r="F14" t="n">
-        <v>5.867810134768883</v>
+        <v>5.824999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>6.267092667943198</v>
+        <v>6.246853956131094</v>
       </c>
       <c r="H14" t="n">
-        <v>6.796228742714516</v>
+        <v>6.819118199903117</v>
       </c>
     </row>
     <row r="15">
@@ -2454,13 +2454,13 @@
         <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>6.655022829612451</v>
+        <v>6.583047424731074</v>
       </c>
       <c r="G15" t="n">
-        <v>6.819912168590496</v>
+        <v>6.698516263439359</v>
       </c>
       <c r="H15" t="n">
-        <v>7.020748537994402</v>
+        <v>6.900139837360185</v>
       </c>
     </row>
     <row r="16">
@@ -2482,13 +2482,13 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>4.477105858498857</v>
+        <v>4.407509507712392</v>
       </c>
       <c r="G16" t="n">
-        <v>5.447938047516743</v>
+        <v>5.481337855009455</v>
       </c>
       <c r="H16" t="n">
-        <v>6.238323917510907</v>
+        <v>6.282784819998072</v>
       </c>
     </row>
     <row r="17">
@@ -2510,13 +2510,13 @@
         <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>4.659168758156628</v>
+        <v>4.564022737736554</v>
       </c>
       <c r="G17" t="n">
-        <v>4.782537555386879</v>
+        <v>4.704556034058134</v>
       </c>
       <c r="H17" t="n">
-        <v>4.87826428304801</v>
+        <v>4.850516014234875</v>
       </c>
     </row>
     <row r="18">
@@ -2538,13 +2538,13 @@
         <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>2.726657362903647</v>
+        <v>2.712659863698741</v>
       </c>
       <c r="G18" t="n">
-        <v>3.1287505843467</v>
+        <v>3.151962644367367</v>
       </c>
       <c r="H18" t="n">
-        <v>3.673135756733777</v>
+        <v>3.734334088493765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>